<commit_message>
fix: invoice excel date format
</commit_message>
<xml_diff>
--- a/examples/invoice.xlsx
+++ b/examples/invoice.xlsx
@@ -1,38 +1,108 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my-projects\invoice-generator\examples\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF076C4-B56B-4BFC-AFEF-6239025DC78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Invoice" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Items" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Invoice" sheetId="1" r:id="rId1"/>
+    <sheet name="Items" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>invoice_number</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>customer</t>
+  </si>
+  <si>
+    <t>Company ABC</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Website development services</t>
+  </si>
+  <si>
+    <t>technical_code</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>unit_price</t>
+  </si>
+  <si>
+    <t>discount_percent</t>
+  </si>
+  <si>
+    <t>PRD-001</t>
+  </si>
+  <si>
+    <t>Product A</t>
+  </si>
+  <si>
+    <t>Product B</t>
+  </si>
+  <si>
+    <t>PRD-003</t>
+  </si>
+  <si>
+    <t>Product C</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,85 +120,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -416,79 +426,53 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>invoice_number</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>10023</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>customer</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Company ABC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Website development services</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>10023</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -497,97 +481,73 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>technical_code</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>unit_price</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>discount_percent</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PRD-001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Product A</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
         <v>2</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>500000</v>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Product B</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
         <v>3</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>250000</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>10</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PRD-003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Product C</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>1000000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update invoice example
</commit_message>
<xml_diff>
--- a/examples/invoice.xlsx
+++ b/examples/invoice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my-projects\invoice-generator\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF076C4-B56B-4BFC-AFEF-6239025DC78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65FDF974-8588-4F80-8EDC-79AB9F94C662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Field</t>
   </si>
@@ -43,15 +43,9 @@
     <t>customer</t>
   </si>
   <si>
-    <t>Company ABC</t>
-  </si>
-  <si>
     <t>description</t>
   </si>
   <si>
-    <t>Website development services</t>
-  </si>
-  <si>
     <t>technical_code</t>
   </si>
   <si>
@@ -64,19 +58,31 @@
     <t>discount_percent</t>
   </si>
   <si>
-    <t>PRD-001</t>
-  </si>
-  <si>
-    <t>Product A</t>
-  </si>
-  <si>
-    <t>Product B</t>
-  </si>
-  <si>
-    <t>PRD-003</t>
-  </si>
-  <si>
-    <t>Product C</t>
+    <t>مرادی جاده بوشهر</t>
+  </si>
+  <si>
+    <t>فاکتور تستی با دیتای تستی</t>
+  </si>
+  <si>
+    <t>منبع هیدرولیک-405مارک</t>
+  </si>
+  <si>
+    <t>گردگیر روی جعبه فرمان (3 عددی)</t>
+  </si>
+  <si>
+    <t>پولی هیدرولیک پرسی (2)</t>
+  </si>
+  <si>
+    <t>پولی هیدرولیک خاری - آیتیپیکوپلاس 2-5</t>
+  </si>
+  <si>
+    <t>سیلندر ترمز چرخ عقب سمند - آذین تنه (مارک) 7</t>
+  </si>
+  <si>
+    <t>رگلاژ چرخ عقب چپ 206 - رسمی</t>
+  </si>
+  <si>
+    <t>رگلاژ چرخ عقب راست 405</t>
   </si>
 </sst>
 </file>
@@ -84,7 +90,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -120,11 +126,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,7 +455,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>10023</v>
+        <v>97628</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -456,7 +463,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -464,15 +471,15 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -482,7 +489,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -494,61 +501,120 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4">
+        <v>8550000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>17011020004</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>500000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3">
-        <v>250000</v>
+        <v>20</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1850000</v>
       </c>
       <c r="E3">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4">
+        <v>17042010001</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
+        <v>11900000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>17042010002</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4">
+        <v>11900000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>556</v>
+      </c>
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1000000</v>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" s="4">
+        <v>4950000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>18011020009</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2450000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>18031020021</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1950000</v>
+      </c>
+      <c r="E8">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>